<commit_message>
Rewrite the prose in plainer language and trim the notes in the notebook
</commit_message>
<xml_diff>
--- a/Task_Sheet_PCA_Formative_2_Pair15.xlsx
+++ b/Task_Sheet_PCA_Formative_2_Pair15.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Data handling, PCA code, plots, benchmarking, GitHub repo setup</t>
+          <t>Dataset, data handling, PCA code, plots, benchmarks, GitHub repo</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -713,7 +713,7 @@
       <c r="A10" s="9" t="n"/>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Chose the dataset: Our World in Data energy data for 54 African countries (2000-2022), checked against the brief (African, 7+ columns, real missing values, text columns)</t>
+          <t>Picked the dataset: Our World in Data energy data for 54 African countries (2000-2022), and checked it against the brief</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -764,7 +764,7 @@
       <c r="A11" s="9" t="n"/>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Data handling: found the missing cells, filled them from each country's own years (sub-region median for the four countries with no GDP), encoded the text columns and log-transformed the skewed ones</t>
+          <t>Data handling: found the blanks, filled them in, turned the text columns into numbers and logged the skewed ones</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>Every step is explained in the notebook.</t>
+          <t>Explained step by step in the notebook.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n"/>
@@ -815,7 +815,7 @@
       <c r="A12" s="9" t="n"/>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>PCA from scratch in numpy: standardization, covariance matrix, eigendecomposition, sorting and projection (Steps 1-7), with checks that each result is correct</t>
+          <t>PCA from scratch in numpy: standardize, covariance, eigendecomposition, sort and project (Steps 1-7), with a check after each step</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>Eigenvalues sum to exactly 19, eigenvectors are orthonormal.</t>
+          <t>Eigenvalues add up to exactly 19 and the eigenvectors are orthonormal.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
@@ -866,7 +866,7 @@
       <c r="A13" s="9" t="n"/>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Explained variance and choosing the number of components from a variance threshold, with scree and cumulative variance plots (Task 2 code)</t>
+          <t>Worked out how many components to keep from the explained variance, with scree and cumulative variance plots (Task 2 code)</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
@@ -917,7 +917,7 @@
       <c r="A14" s="9" t="n"/>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>Before and after PCA plots, component loadings and a chart of the information lost per feature (Step 8)</t>
+          <t>Before and after PCA plots, component loadings and a chart of what information is lost per feature (Step 8)</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
@@ -964,7 +964,7 @@
       <c r="A15" s="9" t="n"/>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>Performance benchmarking for large data: loops vs vectorized, float32 vs float64, chunked covariance and SVD, up to 1,000,000 rows (Task 3)</t>
+          <t>Speed tests for big data: loops vs vectorized, float32 vs float64, chunked covariance and SVD, up to 1,000,000 rows (Task 3)</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
@@ -1011,7 +1011,7 @@
       <c r="A16" s="9" t="n"/>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Wrote the covariance explanation and the three interpretation answers (before/after plot, choice of components and trade-offs, information lost)</t>
+          <t>Wrote the covariance explanation and the three interpretation answers (before/after plot, number of components and trade-offs, what is lost)</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -1062,7 +1062,7 @@
       <c r="A17" s="9" t="n"/>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Ran the notebook in Google Colab and checked every output, then post a short verification note on GitHub</t>
+          <t>Ran the notebook in Google Colab and checked every output, then post a short note on GitHub saying it works</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>Re-ran it in Colab with no errors. The GitHub note is still to post.</t>
+          <t>Ran it in Colab with no errors. Still need to post the GitHub note.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n"/>
@@ -1164,7 +1164,7 @@
       <c r="A19" s="9" t="n"/>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>GitHub: added the how-to-run-in-Colab section and a results summary to the README</t>
+          <t>GitHub: added a how-to-run-in-Colab section and a results summary to the README</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
@@ -1193,7 +1193,7 @@
       <c r="A20" s="9" t="n"/>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>GitHub: wrote data/DATA_DICTIONARY.md covering the 15 features and the sub_region column</t>
+          <t>GitHub: wrote data/DATA_DICTIONARY.md for the 15 features and the sub_region column</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -1222,7 +1222,7 @@
       <c r="A21" s="9" t="n"/>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Final steps: download the Google Doc as a PDF, merge it with the task sheet PDF, final check and submit on Canvas</t>
+          <t>Last steps: download the Google Doc as a PDF, merge it with the task sheet PDF, final check and submit on Canvas</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -1377,12 +1377,12 @@
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>Went through the PCA brief and the rubric together. Agreed who does what: Nelly takes the data, the PCA code, the plots and the benchmarking. Mutoni takes the written answers, the Colab check and the GitHub README and data dictionary.</t>
+          <t>Went through the brief and the rubric together and split the work. Nelly does the data, the PCA code, the plots and the benchmarks. Mutoni does the written answers, the Colab check, and the README and data dictionary.</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>Nelly to find a dataset and build the notebook. Mutoni to start on her parts once the notebook is ready.</t>
+          <t>Nelly finds a dataset and builds the notebook. Mutoni starts her parts once the notebook is ready.</t>
         </is>
       </c>
       <c r="G25" s="9" t="n"/>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>Notebook, GitHub repo and report are done. Mutoni added her written answers, the README and the data dictionary, and ran the notebook in Colab. Went over what's left: the task sheet, the final PDF and submitting.</t>
+          <t>The notebook, repo and report are done. Mutoni added her answers, the README and the data dictionary, and ran the notebook in Colab. We went through what's left: the task sheet, the final PDF and submitting.</t>
         </is>
       </c>
       <c r="F26" s="13" t="inlineStr">

</xml_diff>